<commit_message>
Update CarePath clinic application
</commit_message>
<xml_diff>
--- a/clinic_report.xlsx
+++ b/clinic_report.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Findings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Trends" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Department Revenue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patient Segmentation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Severity by Department" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Key Findings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Monthly Trends" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Department Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Patient Segmentation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Appointment Status" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -150,18 +150,18 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Monthly Diagnosis Volume</a:t>
+              <a:t>Monthly Appointment Volume</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -179,14 +179,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -211,6 +211,21 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -223,6 +238,21 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Appointments</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -238,13 +268,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -267,14 +297,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -326,13 +356,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -356,7 +386,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -393,6 +423,21 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue (EGP)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -408,13 +453,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -437,7 +482,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -465,13 +510,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -495,7 +540,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -547,18 +592,18 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Diagnosis Severity by Department</a:t>
+              <a:t>Appointment Status by Department</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -573,22 +618,22 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Severity by Department'!B1</f>
+              <f>'Appointment Status'!B1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Severity by Department'!$A$2:$A$9</f>
+              <f>'Appointment Status'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Severity by Department'!$B$2:$B$9</f>
+              <f>'Appointment Status'!$B$2:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -597,22 +642,22 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Severity by Department'!C1</f>
+              <f>'Appointment Status'!C1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Severity by Department'!$A$2:$A$9</f>
+              <f>'Appointment Status'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Severity by Department'!$C$2:$C$9</f>
+              <f>'Appointment Status'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -621,22 +666,22 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Severity by Department'!D1</f>
+              <f>'Appointment Status'!D1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Severity by Department'!$A$2:$A$9</f>
+              <f>'Appointment Status'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Severity by Department'!$D$2:$D$9</f>
+              <f>'Appointment Status'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -678,7 +723,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -693,9 +738,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -715,9 +760,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -727,7 +772,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -742,9 +787,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -754,7 +799,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -769,9 +814,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -791,9 +836,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -803,7 +848,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -818,9 +863,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1127,7 +1172,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CLINIC OPERATIONS — KEY FINDINGS (v2 schema)</t>
+          <t>CLINIC OPERATIONS — KEY FINDINGS</t>
         </is>
       </c>
     </row>
@@ -1137,49 +1182,49 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1. Peak diagnosis month: 2025-07</t>
+          <t>1. Peak appointment month: 2025-07</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2. Peak revenue month: 2026-01 (EGP 402,001.35)</t>
+          <t>2. Peak revenue month: 2025-07 (EGP 179,250.84)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3. Highest-revenue department: General Medicine (EGP 1,791,000.20)</t>
+          <t>3. Highest-revenue department: General Medicine (EGP 798,965.18)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4. Largest patient age segment: 60+ (1688 patients)</t>
+          <t>4. Largest patient age segment: 60+ (1734 patients)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5. Most represented city: Tanta (643 patients)</t>
+          <t>5. Most represented city: Tanta (645 patients)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>6. Overdue payments run ~10% of billing records — see 'Payments' sheet for the department breakdown.</t>
+          <t>6. No-show rate averages ~15% overall, with variation across departments — see 'Appointment Status' sheet.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>7. The linear chain (Department -&gt; Doctor -&gt; Patient -&gt; Diagnosis -&gt; Billing -&gt; Lab Tests) makes each patient's full journey traceable end-to-end from a single diagnosis record.</t>
+          <t>7. No single patient/appointment attribute strongly predicts no-shows on its own — a richer feature set (e.g. appointment lead time, past no-show history) would likely improve prediction accuracy.</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1250,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>num_diagnoses</t>
+          <t>num_appointments</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -1226,7 +1271,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>513</v>
+        <v>636</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1234,7 +1279,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>233470.49</v>
+        <v>120992.57</v>
       </c>
     </row>
     <row r="3">
@@ -1244,7 +1289,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>886</v>
+        <v>847</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1252,7 +1297,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>377665.16</v>
+        <v>166053.26</v>
       </c>
     </row>
     <row r="4">
@@ -1262,7 +1307,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>811</v>
+        <v>829</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1270,7 +1315,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>357804.28</v>
+        <v>162312.81</v>
       </c>
     </row>
     <row r="5">
@@ -1280,7 +1325,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>797</v>
+        <v>854</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1288,7 +1333,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>343186.08</v>
+        <v>163385.59</v>
       </c>
     </row>
     <row r="6">
@@ -1298,7 +1343,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>798</v>
+        <v>849</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1306,7 +1351,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>340642.11</v>
+        <v>169376.11</v>
       </c>
     </row>
     <row r="7">
@@ -1316,7 +1361,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>713</v>
+        <v>732</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1324,7 +1369,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>316196.19</v>
+        <v>147069.92</v>
       </c>
     </row>
     <row r="8">
@@ -1334,7 +1379,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>851</v>
+        <v>865</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1342,7 +1387,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>384341.34</v>
+        <v>170913.66</v>
       </c>
     </row>
     <row r="9">
@@ -1352,7 +1397,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>788</v>
+        <v>809</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1360,7 +1405,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>346668.64</v>
+        <v>158754.32</v>
       </c>
     </row>
     <row r="10">
@@ -1370,7 +1415,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>829</v>
+        <v>869</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1378,7 +1423,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>361743.68</v>
+        <v>165805.04</v>
       </c>
     </row>
     <row r="11">
@@ -1388,7 +1433,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>799</v>
+        <v>775</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1396,7 +1441,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>343558.29</v>
+        <v>151392.09</v>
       </c>
     </row>
     <row r="12">
@@ -1406,7 +1451,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>900</v>
+        <v>914</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1414,7 +1459,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>389349.57</v>
+        <v>179250.84</v>
       </c>
     </row>
     <row r="13">
@@ -1424,7 +1469,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>876</v>
+        <v>863</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1432,7 +1477,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>391004.36</v>
+        <v>172086.72</v>
       </c>
     </row>
     <row r="14">
@@ -1442,7 +1487,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>797</v>
+        <v>827</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1450,7 +1495,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>354437.08</v>
+        <v>157748.73</v>
       </c>
     </row>
     <row r="15">
@@ -1460,7 +1505,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>841</v>
+        <v>785</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1468,7 +1513,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>375447.06</v>
+        <v>159179.77</v>
       </c>
     </row>
     <row r="16">
@@ -1478,7 +1523,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>871</v>
+        <v>832</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1486,7 +1531,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>380829.89</v>
+        <v>165246.2</v>
       </c>
     </row>
     <row r="17">
@@ -1496,7 +1541,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>857</v>
+        <v>906</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1504,7 +1549,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>381076.09</v>
+        <v>176084.65</v>
       </c>
     </row>
     <row r="18">
@@ -1514,7 +1559,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>889</v>
+        <v>824</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1522,7 +1567,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>402001.35</v>
+        <v>156038.32</v>
       </c>
     </row>
     <row r="19">
@@ -1532,7 +1577,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>778</v>
+        <v>756</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1540,7 +1585,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>352425.57</v>
+        <v>143974.95</v>
       </c>
     </row>
     <row r="20">
@@ -1550,7 +1595,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>849</v>
+        <v>836</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1558,7 +1603,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>364912.58</v>
+        <v>157254.36</v>
       </c>
     </row>
     <row r="21">
@@ -1568,7 +1613,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>878</v>
+        <v>819</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1576,7 +1621,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>387785.86</v>
+        <v>166235.56</v>
       </c>
     </row>
     <row r="22">
@@ -1586,7 +1631,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>816</v>
+        <v>852</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1594,7 +1639,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>366758.6</v>
+        <v>166833</v>
       </c>
     </row>
     <row r="23">
@@ -1604,7 +1649,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>832</v>
+        <v>805</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1612,7 +1657,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>362526.1</v>
+        <v>150582.59</v>
       </c>
     </row>
     <row r="24">
@@ -1622,7 +1667,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>864</v>
+        <v>828</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1630,7 +1675,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>387430.88</v>
+        <v>160328.1</v>
       </c>
     </row>
     <row r="25">
@@ -1640,7 +1685,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>839</v>
+        <v>824</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1648,7 +1693,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>379985.44</v>
+        <v>157332.9</v>
       </c>
     </row>
     <row r="26">
@@ -1658,7 +1703,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>328</v>
+        <v>264</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1666,7 +1711,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>146254.72</v>
+        <v>56939.84</v>
       </c>
     </row>
   </sheetData>
@@ -1703,7 +1748,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1791000.2</v>
+        <v>798965.1800000001</v>
       </c>
     </row>
     <row r="3">
@@ -1713,27 +1758,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1438119.76</v>
+        <v>625948.65</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dermatology</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1434831.92</v>
+        <v>548657.33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>Dermatology</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1021632.1</v>
+        <v>497830.64</v>
       </c>
     </row>
     <row r="6">
@@ -1743,27 +1788,27 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1005010.86</v>
+        <v>478168</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ENT</t>
+          <t>Dentistry</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>818719.62</v>
+        <v>351390.02</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dentistry</t>
+          <t>ENT</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>783095.34</v>
+        <v>317825.01</v>
       </c>
     </row>
     <row r="9">
@@ -1773,7 +1818,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>535091.61</v>
+        <v>282387.07</v>
       </c>
     </row>
   </sheetData>
@@ -1820,7 +1865,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1688</v>
+        <v>1734</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1828,7 +1873,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="3">
@@ -1838,7 +1883,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1251</v>
+        <v>1229</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1846,7 +1891,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>638</v>
+        <v>642</v>
       </c>
     </row>
     <row r="4">
@@ -1856,7 +1901,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1116</v>
+        <v>1079</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1864,7 +1909,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="5">
@@ -1874,25 +1919,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>945</v>
+        <v>958</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Alexandria</t>
+          <t>Aswan</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="6">
       <c r="D6" t="inlineStr">
         <is>
-          <t>Aswan</t>
+          <t>Alexandria</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>633</v>
+        <v>629</v>
       </c>
     </row>
     <row r="7">
@@ -1912,7 +1957,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>626</v>
+        <v>622</v>
       </c>
     </row>
     <row r="9">
@@ -1922,7 +1967,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
   </sheetData>
@@ -1948,17 +1993,17 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Mild</t>
+          <t>Attended</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Cancelled</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Severe</t>
+          <t>No-show</t>
         </is>
       </c>
     </row>
@@ -1969,13 +2014,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1335</v>
+        <v>1848</v>
       </c>
       <c r="C2" t="n">
-        <v>767</v>
+        <v>258</v>
       </c>
       <c r="D2" t="n">
-        <v>171</v>
+        <v>382</v>
       </c>
     </row>
     <row r="3">
@@ -1985,13 +2030,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1000</v>
+        <v>1356</v>
       </c>
       <c r="C3" t="n">
-        <v>582</v>
+        <v>157</v>
       </c>
       <c r="D3" t="n">
-        <v>150</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4">
@@ -2001,13 +2046,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1897</v>
+        <v>1925</v>
       </c>
       <c r="C4" t="n">
-        <v>1083</v>
+        <v>228</v>
       </c>
       <c r="D4" t="n">
-        <v>265</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5">
@@ -2017,13 +2062,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1128</v>
+        <v>1230</v>
       </c>
       <c r="C5" t="n">
-        <v>653</v>
+        <v>156</v>
       </c>
       <c r="D5" t="n">
-        <v>130</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6">
@@ -2033,13 +2078,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2374</v>
+        <v>3071</v>
       </c>
       <c r="C6" t="n">
-        <v>1301</v>
+        <v>396</v>
       </c>
       <c r="D6" t="n">
-        <v>347</v>
+        <v>567</v>
       </c>
     </row>
     <row r="7">
@@ -2049,13 +2094,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>726</v>
+        <v>1097</v>
       </c>
       <c r="C7" t="n">
-        <v>400</v>
+        <v>144</v>
       </c>
       <c r="D7" t="n">
-        <v>86</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8">
@@ -2065,13 +2110,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1930</v>
+        <v>2402</v>
       </c>
       <c r="C8" t="n">
-        <v>1128</v>
+        <v>339</v>
       </c>
       <c r="D8" t="n">
-        <v>279</v>
+        <v>443</v>
       </c>
     </row>
     <row r="9">
@@ -2081,13 +2126,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1329</v>
+        <v>2114</v>
       </c>
       <c r="C9" t="n">
-        <v>736</v>
+        <v>293</v>
       </c>
       <c r="D9" t="n">
-        <v>203</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>